<commit_message>
BRO: Default wordt geen SKOS gegenereerd
</commit_message>
<xml_diff>
--- a/src/main/resources/input/BRO/props/BRO.xlsx
+++ b/src/main/resources/input/BRO/props/BRO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\gitprojects\Imvertor-Maven\src\main\resources\input\BRO\props\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3124F50-7524-4279-8254-788E4FA19634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5D4CE8-0142-427F-9640-375199F0CE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="20057" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="387">
   <si>
     <t>Name</t>
   </si>
@@ -2946,21 +2946,6 @@
         <v>14</v>
       </c>
       <c r="G39" s="24"/>
-      <c r="H39" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="I39" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="J39" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="K39" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="L39" s="23" t="s">
-        <v>4</v>
-      </c>
       <c r="M39" s="24"/>
       <c r="S39" s="24"/>
     </row>

</xml_diff>